<commit_message>
Update assumptions.xlsx via admin panel
</commit_message>
<xml_diff>
--- a/data/assumptions.xlsx
+++ b/data/assumptions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ekosltd-my.sharepoint.com/personal/alessia_biris_ekos_co_uk/Documents/TCL/code_dashboard/v2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="8_{FA218BAD-3EBA-47B7-9DEF-468792D266E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FA303A8-BBEE-4BD1-8454-7FFFA21B5672}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="8_{FA218BAD-3EBA-47B7-9DEF-468792D266E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BEDB1A4-74A1-481E-B850-1F6C3745C7BE}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="13" xr2:uid="{5C67809F-44A3-4AFA-BBD2-6581972C325D}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="17" xr2:uid="{5C67809F-44A3-4AFA-BBD2-6581972C325D}"/>
   </bookViews>
   <sheets>
     <sheet name="general_parameters" sheetId="1" r:id="rId1"/>
@@ -1622,20 +1622,13 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color indexed="64"/>
         </left>
         <right style="medium">
           <color indexed="64"/>
         </right>
-        <top style="thin">
+        <top style="medium">
           <color indexed="64"/>
         </top>
         <bottom style="medium">
@@ -1729,6 +1722,42 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="170" formatCode="0.0%"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1782,13 +1811,20 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <left style="medium">
           <color indexed="64"/>
         </left>
         <right style="medium">
           <color indexed="64"/>
         </right>
-        <top style="medium">
+        <top style="thin">
           <color indexed="64"/>
         </top>
         <bottom style="medium">
@@ -1844,12 +1880,19 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <color rgb="FF666666"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="169" formatCode="0.0\x"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1877,12 +1920,19 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <color rgb="FF666666"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0%;[Red]\(0.0%\);\-"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1912,13 +1962,19 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="170" formatCode="0.0%"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <color rgb="FF666666"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0%;[Red]\(0.0%\);\-"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1948,12 +2004,89 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <color rgb="FF666666"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0%;[Red]\(0.0%\);\-"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Avenir Next LT Pro"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="thin">
@@ -1993,6 +2126,31 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF666666"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
@@ -2001,22 +2159,28 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDCE6F1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -4845,19 +5009,12 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FF666666"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="169" formatCode="0.0\x"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <color theme="1"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -4885,19 +5042,12 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FF666666"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0%;[Red]\(0.0%\);\-"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <color theme="1"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -4927,131 +5077,12 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FF666666"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0%;[Red]\(0.0%\);\-"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0%;[Red]\(0.0%\);\-"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
         <color theme="1"/>
         <name val="Avenir Next LT Pro"/>
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="thin">
@@ -5091,31 +5122,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF666666"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
@@ -5124,28 +5130,22 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Avenir Next LT Pro"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFDCE6F1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -5170,86 +5170,82 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5C45BCAE-2920-4A62-AF02-18762D92BA91}" name="general_parameters" displayName="general_parameters" ref="A1:D8" totalsRowShown="0" headerRowDxfId="139" headerRowBorderDxfId="138" tableBorderDxfId="137" totalsRowBorderDxfId="136">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5C45BCAE-2920-4A62-AF02-18762D92BA91}" name="general_parameters" displayName="general_parameters" ref="A1:D8" totalsRowShown="0" headerRowDxfId="143" headerRowBorderDxfId="142" tableBorderDxfId="141" totalsRowBorderDxfId="140">
   <autoFilter ref="A1:D8" xr:uid="{5C45BCAE-2920-4A62-AF02-18762D92BA91}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{BF4A73EA-A313-4283-BE5C-5B9F6C2039F3}" name="Parameter" dataDxfId="135"/>
+    <tableColumn id="1" xr3:uid="{BF4A73EA-A313-4283-BE5C-5B9F6C2039F3}" name="Parameter" dataDxfId="139"/>
     <tableColumn id="2" xr3:uid="{2168A1D6-1F00-420A-AE49-628879EF67CF}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{EE2AD78A-DCFF-47D8-A4FD-47301D7A564F}" name="Units" dataDxfId="134"/>
-    <tableColumn id="4" xr3:uid="{F7910500-F089-4E59-9AC8-5734EF06B071}" name="Source / note" dataDxfId="133"/>
+    <tableColumn id="3" xr3:uid="{EE2AD78A-DCFF-47D8-A4FD-47301D7A564F}" name="Units" dataDxfId="138"/>
+    <tableColumn id="4" xr3:uid="{F7910500-F089-4E59-9AC8-5734EF06B071}" name="Source / note" dataDxfId="137"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{14481E30-4492-4DED-8E9A-2EC2D68F1FBA}" name="household_spend" displayName="household_spend" ref="A1:E11" totalsRowShown="0" headerRowDxfId="52" dataDxfId="50" headerRowBorderDxfId="51" tableBorderDxfId="49" totalsRowBorderDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{14481E30-4492-4DED-8E9A-2EC2D68F1FBA}" name="household_spend" displayName="household_spend" ref="A1:E11" totalsRowShown="0" headerRowDxfId="56" dataDxfId="54" headerRowBorderDxfId="55" tableBorderDxfId="53" totalsRowBorderDxfId="52">
   <autoFilter ref="A1:E11" xr:uid="{14481E30-4492-4DED-8E9A-2EC2D68F1FBA}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{9A4690EE-FA56-405E-A30D-875570657134}" name="Typology / tenure" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{E91F277E-06CE-4EDB-8543-29E44E82DEA7}" name="Upper" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{1EAAF470-471D-4B0C-A575-DFBD58AEA1B8}" name="Central" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{57C7CBC2-465E-4D9C-862C-8B255FF6A5B2}" name="Lower" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{2AC2BF98-5348-4DE0-93F2-91C9D65F223E}" name="Units" dataDxfId="43"/>
+    <tableColumn id="1" xr3:uid="{9A4690EE-FA56-405E-A30D-875570657134}" name="Typology / tenure" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{E91F277E-06CE-4EDB-8543-29E44E82DEA7}" name="Upper" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{1EAAF470-471D-4B0C-A575-DFBD58AEA1B8}" name="Central" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{57C7CBC2-465E-4D9C-862C-8B255FF6A5B2}" name="Lower" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{2AC2BF98-5348-4DE0-93F2-91C9D65F223E}" name="Units" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{10CAE23F-64C2-446D-8AC7-2420C696FBA2}" name="additionality_mappings" displayName="additionality_mappings" ref="A1:F16" totalsRowShown="0" headerRowDxfId="150" dataDxfId="148" headerRowBorderDxfId="149" tableBorderDxfId="147" totalsRowBorderDxfId="146">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{10CAE23F-64C2-446D-8AC7-2420C696FBA2}" name="additionality_mappings" displayName="additionality_mappings" ref="A1:F16" totalsRowShown="0" headerRowDxfId="46" dataDxfId="44" headerRowBorderDxfId="45" tableBorderDxfId="43" totalsRowBorderDxfId="42">
   <autoFilter ref="A1:F16" xr:uid="{10CAE23F-64C2-446D-8AC7-2420C696FBA2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{E3A723FA-457B-4EFE-9E92-EB013E337B59}" name="Group" dataDxfId="145"/>
-    <tableColumn id="2" xr3:uid="{02D51F27-6686-45C8-B830-EE4683B203DE}" name="Scenario" dataDxfId="144"/>
-    <tableColumn id="3" xr3:uid="{141761B2-F5F5-4B9A-8B3E-DC8AC7A74CBC}" name="Deadweight" dataDxfId="143"/>
-    <tableColumn id="4" xr3:uid="{73079F49-39D1-41A2-AF81-9562C0ADE495}" name="Displacement" dataDxfId="142"/>
-    <tableColumn id="5" xr3:uid="{BF1D37EB-AE48-4C08-9998-896BCDE53C45}" name="Leakage" dataDxfId="141"/>
-    <tableColumn id="6" xr3:uid="{343EC36C-1426-4634-AD97-7726BDCCA977}" name="Multiplier" dataDxfId="140"/>
+    <tableColumn id="1" xr3:uid="{E3A723FA-457B-4EFE-9E92-EB013E337B59}" name="Group" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{02D51F27-6686-45C8-B830-EE4683B203DE}" name="Scenario" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{141761B2-F5F5-4B9A-8B3E-DC8AC7A74CBC}" name="Deadweight" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{73079F49-39D1-41A2-AF81-9562C0ADE495}" name="Displacement" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{BF1D37EB-AE48-4C08-9998-896BCDE53C45}" name="Leakage" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{343EC36C-1426-4634-AD97-7726BDCCA977}" name="Multiplier" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{B1ED9103-DDDE-47B1-8810-5356D0BC801A}" name="discounting" displayName="discounting" ref="A1:D3" totalsRowShown="0" headerRowDxfId="42" headerRowBorderDxfId="41" tableBorderDxfId="40" totalsRowBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{B1ED9103-DDDE-47B1-8810-5356D0BC801A}" name="discounting" displayName="discounting" ref="A1:D3" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33" totalsRowBorderDxfId="32">
   <autoFilter ref="A1:D3" xr:uid="{B1ED9103-DDDE-47B1-8810-5356D0BC801A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C9D1B6E6-554B-4728-999B-F79940D1548F}" name="Parameter" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{9CC8EED5-22B9-4B6C-ABA0-C94CA361A8EB}" name="Value" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{DF9EDA1C-294C-452B-BFF2-26FBD630BCD3}" name="Unit" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{D5D8E8F0-51CC-4FDB-ABC4-1CE5C67CF3DC}" name="Source" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{C9D1B6E6-554B-4728-999B-F79940D1548F}" name="Parameter" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{9CC8EED5-22B9-4B6C-ABA0-C94CA361A8EB}" name="Value" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{DF9EDA1C-294C-452B-BFF2-26FBD630BCD3}" name="Unit" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{D5D8E8F0-51CC-4FDB-ABC4-1CE5C67CF3DC}" name="Source" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{6423D1D0-30EB-48F7-8293-4EDC0FFE06C1}" name="discounting_by_impact" displayName="discounting_by_impact" ref="A1:D4" totalsRowShown="0" headerRowDxfId="34" headerRowBorderDxfId="33" tableBorderDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{6423D1D0-30EB-48F7-8293-4EDC0FFE06C1}" name="discounting_by_impact" displayName="discounting_by_impact" ref="A1:D4" totalsRowShown="0" headerRowDxfId="27" headerRowBorderDxfId="26" tableBorderDxfId="25">
   <autoFilter ref="A1:D4" xr:uid="{6423D1D0-30EB-48F7-8293-4EDC0FFE06C1}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{BAA839D6-42E3-4FD9-8386-2108D73EF939}" name="Impact" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{BAA839D6-42E3-4FD9-8386-2108D73EF939}" name="Impact" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{34EDF934-C8FE-4FFD-9217-6E193C221B78}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{6516570E-DCB9-4F5C-8D62-991AA6C746A7}" name="Unit" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{B4F1FF20-BFB8-46B8-A719-D89B829DB05B}" name="Notes" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{6516570E-DCB9-4F5C-8D62-991AA6C746A7}" name="Unit" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{B4F1FF20-BFB8-46B8-A719-D89B829DB05B}" name="Notes" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{4EB637CF-069E-41D0-AB72-259C07748F40}" name="land_infra_mult" displayName="land_infra_mult" ref="A1:D9" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26" totalsRowBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{4EB637CF-069E-41D0-AB72-259C07748F40}" name="land_infra_mult" displayName="land_infra_mult" ref="A1:D9" totalsRowShown="0" headerRowDxfId="150" headerRowBorderDxfId="149" tableBorderDxfId="148" totalsRowBorderDxfId="147">
   <autoFilter ref="A1:D9" xr:uid="{4EB637CF-069E-41D0-AB72-259C07748F40}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{7FD0A6E6-1B0A-4FC7-81EC-4DD560B478DC}" name="Parameter" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{7FD0A6E6-1B0A-4FC7-81EC-4DD560B478DC}" name="Parameter" dataDxfId="146"/>
     <tableColumn id="2" xr3:uid="{A7B1CC4E-78DF-4D14-A750-3E88F52FAF2A}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{2E3AE3B4-C3F9-4F53-873A-03E831ED79B8}" name="Unit" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{4BF2B9CD-2B84-4D85-BBB6-91888AED0426}" name="Notes" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{2E3AE3B4-C3F9-4F53-873A-03E831ED79B8}" name="Unit" dataDxfId="145"/>
+    <tableColumn id="4" xr3:uid="{4BF2B9CD-2B84-4D85-BBB6-91888AED0426}" name="Notes" dataDxfId="144"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5304,118 +5300,118 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0E3C03BC-9795-4A32-BE15-F23695000642}" name="dwellingbytypology" displayName="dwellingbytypology" ref="A1:H6" totalsRowShown="0" headerRowDxfId="132" dataDxfId="130" headerRowBorderDxfId="131" tableBorderDxfId="129" totalsRowBorderDxfId="128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0E3C03BC-9795-4A32-BE15-F23695000642}" name="dwellingbytypology" displayName="dwellingbytypology" ref="A1:H6" totalsRowShown="0" headerRowDxfId="136" dataDxfId="134" headerRowBorderDxfId="135" tableBorderDxfId="133" totalsRowBorderDxfId="132">
   <autoFilter ref="A1:H6" xr:uid="{0E3C03BC-9795-4A32-BE15-F23695000642}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{AF5B1002-ACF0-443F-BA91-D855456C8E2D}" name="Typology" dataDxfId="127"/>
-    <tableColumn id="2" xr3:uid="{4552E384-A064-4D7E-B638-6DC25252B385}" name="Floorspace m2" dataDxfId="126"/>
-    <tableColumn id="3" xr3:uid="{E22864B2-160F-4F3D-9491-0A60A9310C41}" name="Persons Per Dwelling - Private" dataDxfId="125"/>
-    <tableColumn id="4" xr3:uid="{0377E05F-6D73-4E82-AD3D-2AA209958578}" name="Persons Per Dwelling - Social/affordable" dataDxfId="124"/>
-    <tableColumn id="5" xr3:uid="{3D93BA7B-360E-4A20-BB94-AFEC8DAB2F05}" name="Council Tax per unit" dataDxfId="123"/>
-    <tableColumn id="6" xr3:uid="{E1042461-7B4B-4E4A-96C1-EA75409C533A}" name="Rent per social/MMR unit" dataDxfId="122"/>
-    <tableColumn id="7" xr3:uid="{56B6CFB9-570D-4CC0-9162-B0D0FCE94F69}" name="Private disposable income" dataDxfId="121"/>
-    <tableColumn id="8" xr3:uid="{CA5B102B-23EE-4F5D-853D-87DFD7D74ACA}" name="Social/affordable disposable income" dataDxfId="120"/>
+    <tableColumn id="1" xr3:uid="{AF5B1002-ACF0-443F-BA91-D855456C8E2D}" name="Typology" dataDxfId="131"/>
+    <tableColumn id="2" xr3:uid="{4552E384-A064-4D7E-B638-6DC25252B385}" name="Floorspace m2" dataDxfId="130"/>
+    <tableColumn id="3" xr3:uid="{E22864B2-160F-4F3D-9491-0A60A9310C41}" name="Persons Per Dwelling - Private" dataDxfId="129"/>
+    <tableColumn id="4" xr3:uid="{0377E05F-6D73-4E82-AD3D-2AA209958578}" name="Persons Per Dwelling - Social/affordable" dataDxfId="128"/>
+    <tableColumn id="5" xr3:uid="{3D93BA7B-360E-4A20-BB94-AFEC8DAB2F05}" name="Council Tax per unit" dataDxfId="127"/>
+    <tableColumn id="6" xr3:uid="{E1042461-7B4B-4E4A-96C1-EA75409C533A}" name="Rent per social/MMR unit" dataDxfId="126"/>
+    <tableColumn id="7" xr3:uid="{56B6CFB9-570D-4CC0-9162-B0D0FCE94F69}" name="Private disposable income" dataDxfId="125"/>
+    <tableColumn id="8" xr3:uid="{CA5B102B-23EE-4F5D-853D-87DFD7D74ACA}" name="Social/affordable disposable income" dataDxfId="124"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{5D2D2174-90B9-463F-9330-0CCD3522FDE1}" name="pop_employ" displayName="pop_employ" ref="A1:E6" totalsRowShown="0" headerRowDxfId="119" headerRowBorderDxfId="118" tableBorderDxfId="117" totalsRowBorderDxfId="116">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{5D2D2174-90B9-463F-9330-0CCD3522FDE1}" name="pop_employ" displayName="pop_employ" ref="A1:E6" totalsRowShown="0" headerRowDxfId="123" headerRowBorderDxfId="122" tableBorderDxfId="121" totalsRowBorderDxfId="120">
   <autoFilter ref="A1:E6" xr:uid="{5D2D2174-90B9-463F-9330-0CCD3522FDE1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{947CE13C-D8BA-437F-95E3-C118D991F51E}" name="Parameter" dataDxfId="115"/>
-    <tableColumn id="2" xr3:uid="{07D50781-49CC-4BF6-8A8F-30D3D0C13A42}" name="Private" dataDxfId="114"/>
-    <tableColumn id="3" xr3:uid="{9642AD60-1B5A-4683-8E0B-12D1FE0BEBCA}" name="Social/affordable" dataDxfId="113"/>
-    <tableColumn id="5" xr3:uid="{E72D4F67-11C4-42E3-B5A3-627689ABEEC2}" name="Older person" dataDxfId="112"/>
-    <tableColumn id="4" xr3:uid="{D8D5E346-3E52-4B56-B72E-C2C8E3B487BA}" name="Units" dataDxfId="111"/>
+    <tableColumn id="1" xr3:uid="{947CE13C-D8BA-437F-95E3-C118D991F51E}" name="Parameter" dataDxfId="119"/>
+    <tableColumn id="2" xr3:uid="{07D50781-49CC-4BF6-8A8F-30D3D0C13A42}" name="Private" dataDxfId="118"/>
+    <tableColumn id="3" xr3:uid="{9642AD60-1B5A-4683-8E0B-12D1FE0BEBCA}" name="Social/affordable" dataDxfId="117"/>
+    <tableColumn id="5" xr3:uid="{E72D4F67-11C4-42E3-B5A3-627689ABEEC2}" name="Older person" dataDxfId="116"/>
+    <tableColumn id="4" xr3:uid="{D8D5E346-3E52-4B56-B72E-C2C8E3B487BA}" name="Units" dataDxfId="115"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{79CADA8C-6739-4499-8318-8C1A1D43CE67}" name="transport_modal" displayName="transport_modal" ref="A1:H9" totalsRowShown="0" headerRowDxfId="110" dataDxfId="108" headerRowBorderDxfId="109" tableBorderDxfId="107" totalsRowBorderDxfId="106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{79CADA8C-6739-4499-8318-8C1A1D43CE67}" name="transport_modal" displayName="transport_modal" ref="A1:H9" totalsRowShown="0" headerRowDxfId="114" dataDxfId="112" headerRowBorderDxfId="113" tableBorderDxfId="111" totalsRowBorderDxfId="110">
   <autoFilter ref="A1:H9" xr:uid="{79CADA8C-6739-4499-8318-8C1A1D43CE67}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{51D80002-D764-4804-8EC7-BF057B59E144}" name="Mode" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{632F4F89-D565-43F4-8508-41B297AC72E4}" name="Baseline share" dataDxfId="104"/>
-    <tableColumn id="3" xr3:uid="{F88145F9-8928-434C-8CDB-20D90AA0024C}" name="TCL Good" dataDxfId="103"/>
-    <tableColumn id="4" xr3:uid="{B0EC6125-F09D-4332-8FAF-A316F08C437C}" name="TCL Average" dataDxfId="102"/>
-    <tableColumn id="5" xr3:uid="{5AF3B7FB-6119-4BB3-BE48-1C87DAEBA045}" name="TCL Limited" dataDxfId="101"/>
-    <tableColumn id="6" xr3:uid="{28476781-DBA7-44F7-8DFF-F6C7E20BF879}" name="Baseline km" dataDxfId="100"/>
-    <tableColumn id="7" xr3:uid="{15EB3372-9D4F-46B3-A45C-B008382479FA}" name="Emission factor kgCO2e/pkm" dataDxfId="99"/>
-    <tableColumn id="8" xr3:uid="{7C2A1136-FFE8-4A44-AC30-D20CEB0F77DF}" name="Speed km/h" dataDxfId="98"/>
+    <tableColumn id="1" xr3:uid="{51D80002-D764-4804-8EC7-BF057B59E144}" name="Mode" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{632F4F89-D565-43F4-8508-41B297AC72E4}" name="Baseline share" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{F88145F9-8928-434C-8CDB-20D90AA0024C}" name="TCL Good" dataDxfId="107"/>
+    <tableColumn id="4" xr3:uid="{B0EC6125-F09D-4332-8FAF-A316F08C437C}" name="TCL Average" dataDxfId="106"/>
+    <tableColumn id="5" xr3:uid="{5AF3B7FB-6119-4BB3-BE48-1C87DAEBA045}" name="TCL Limited" dataDxfId="105"/>
+    <tableColumn id="6" xr3:uid="{28476781-DBA7-44F7-8DFF-F6C7E20BF879}" name="Baseline km" dataDxfId="104"/>
+    <tableColumn id="7" xr3:uid="{15EB3372-9D4F-46B3-A45C-B008382479FA}" name="Emission factor kgCO2e/pkm" dataDxfId="103"/>
+    <tableColumn id="8" xr3:uid="{7C2A1136-FFE8-4A44-AC30-D20CEB0F77DF}" name="Speed km/h" dataDxfId="102"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B5EB96F9-732E-4614-BCD1-33C1639E5F61}" name="carbon" displayName="carbon" ref="A1:F4" totalsRowShown="0" headerRowDxfId="97" dataDxfId="95" headerRowBorderDxfId="96" tableBorderDxfId="94" totalsRowBorderDxfId="93">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B5EB96F9-732E-4614-BCD1-33C1639E5F61}" name="carbon" displayName="carbon" ref="A1:F4" totalsRowShown="0" headerRowDxfId="101" dataDxfId="99" headerRowBorderDxfId="100" tableBorderDxfId="98" totalsRowBorderDxfId="97">
   <autoFilter ref="A1:F4" xr:uid="{B5EB96F9-732E-4614-BCD1-33C1639E5F61}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{80B2580A-D788-4184-8B9B-91481871C1B1}" name="Development type" dataDxfId="92"/>
-    <tableColumn id="2" xr3:uid="{E2B4663C-5E14-40B1-B0E0-9F536D5994B1}" name="Low upfront" dataDxfId="91"/>
-    <tableColumn id="3" xr3:uid="{4F8B9403-C34D-4A52-AFD9-86BB230C316D}" name="Medium upfront" dataDxfId="90"/>
-    <tableColumn id="4" xr3:uid="{148042E5-61B0-4045-9632-78DA909DE42D}" name="High upfront" dataDxfId="89"/>
-    <tableColumn id="5" xr3:uid="{8A4AFD31-51B7-45FE-8D58-B6C8F3E1E731}" name="Baseline comparator" dataDxfId="88"/>
-    <tableColumn id="6" xr3:uid="{C11B7004-AD50-4B91-A6AC-2CD2E104AC48}" name="End of life factor" dataDxfId="87"/>
+    <tableColumn id="1" xr3:uid="{80B2580A-D788-4184-8B9B-91481871C1B1}" name="Development type" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{E2B4663C-5E14-40B1-B0E0-9F536D5994B1}" name="Low upfront" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{4F8B9403-C34D-4A52-AFD9-86BB230C316D}" name="Medium upfront" dataDxfId="94"/>
+    <tableColumn id="4" xr3:uid="{148042E5-61B0-4045-9632-78DA909DE42D}" name="High upfront" dataDxfId="93"/>
+    <tableColumn id="5" xr3:uid="{8A4AFD31-51B7-45FE-8D58-B6C8F3E1E731}" name="Baseline comparator" dataDxfId="92"/>
+    <tableColumn id="6" xr3:uid="{C11B7004-AD50-4B91-A6AC-2CD2E104AC48}" name="End of life factor" dataDxfId="91"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{AC749976-DD17-482A-9FD7-9196F207272A}" name="environ_wellbeingTable6" displayName="environ_wellbeingTable6" ref="A1:E6" totalsRowShown="0" headerRowDxfId="86" headerRowBorderDxfId="85" tableBorderDxfId="84" totalsRowBorderDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{AC749976-DD17-482A-9FD7-9196F207272A}" name="environ_wellbeingTable6" displayName="environ_wellbeingTable6" ref="A1:E6" totalsRowShown="0" headerRowDxfId="90" headerRowBorderDxfId="89" tableBorderDxfId="88" totalsRowBorderDxfId="87">
   <autoFilter ref="A1:E6" xr:uid="{AC749976-DD17-482A-9FD7-9196F207272A}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{04476D43-8F73-422A-9656-FA2B9CD22585}" name="Parameter" dataDxfId="82"/>
-    <tableColumn id="2" xr3:uid="{76480CDF-9E60-4089-A0A3-B5493DDC105F}" name="Lower scale impact" dataDxfId="81"/>
+    <tableColumn id="1" xr3:uid="{04476D43-8F73-422A-9656-FA2B9CD22585}" name="Parameter" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{76480CDF-9E60-4089-A0A3-B5493DDC105F}" name="Lower scale impact" dataDxfId="85"/>
     <tableColumn id="3" xr3:uid="{AB078BD6-DFAE-44D5-A871-78C491E01176}" name="Central impact"/>
     <tableColumn id="4" xr3:uid="{75FA526C-FBEE-4599-B606-702D6554E485}" name="Higher scale impact"/>
-    <tableColumn id="5" xr3:uid="{0BDF18F5-C495-4B11-AD1B-3043B7B15F46}" name="Units" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{0BDF18F5-C495-4B11-AD1B-3043B7B15F46}" name="Units" dataDxfId="84"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{DC131DAF-A5A6-4609-9BBD-D774FD2E423D}" name="active_travel" displayName="active_travel" ref="A1:G4" totalsRowShown="0" headerRowDxfId="79" dataDxfId="77" headerRowBorderDxfId="78" tableBorderDxfId="76" totalsRowBorderDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{DC131DAF-A5A6-4609-9BBD-D774FD2E423D}" name="active_travel" displayName="active_travel" ref="A1:G4" totalsRowShown="0" headerRowDxfId="83" dataDxfId="81" headerRowBorderDxfId="82" tableBorderDxfId="80" totalsRowBorderDxfId="79">
   <autoFilter ref="A1:G4" xr:uid="{DC131DAF-A5A6-4609-9BBD-D774FD2E423D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{AD78C056-5CC9-4CD9-B25A-9E1FDA7619ED}" name="Accessibility" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{DDB6924C-0BED-4161-92F2-8EF3A236C4E5}" name="Walking uplift" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{9C68EE70-0111-4A45-8C9E-3C0000BE8EB3}" name="Cycling uplift" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{727BFA19-FC13-457E-A671-2032BFC507A9}" name="Minutes uplift" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{4EF746B4-929E-4ADE-9844-064C65AA8AF6}" name="Baseline meeting 150 mins (high deprivation)" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{A508C7D2-8286-46AA-AE93-0CFD202BABC6}" name="Baseline meeting 150 mins (average deprivation)" dataDxfId="69"/>
-    <tableColumn id="7" xr3:uid="{DA5F9070-A695-4818-AAC9-61F124AC7F92}" name="Baseline meeting 150 mins (low deprivation)" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{AD78C056-5CC9-4CD9-B25A-9E1FDA7619ED}" name="Accessibility" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{DDB6924C-0BED-4161-92F2-8EF3A236C4E5}" name="Walking uplift" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{9C68EE70-0111-4A45-8C9E-3C0000BE8EB3}" name="Cycling uplift" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{727BFA19-FC13-457E-A671-2032BFC507A9}" name="Minutes uplift" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{4EF746B4-929E-4ADE-9844-064C65AA8AF6}" name="Baseline meeting 150 mins (high deprivation)" dataDxfId="74"/>
+    <tableColumn id="6" xr3:uid="{A508C7D2-8286-46AA-AE93-0CFD202BABC6}" name="Baseline meeting 150 mins (average deprivation)" dataDxfId="73"/>
+    <tableColumn id="7" xr3:uid="{DA5F9070-A695-4818-AAC9-61F124AC7F92}" name="Baseline meeting 150 mins (low deprivation)" dataDxfId="72"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EF810BE9-7C6F-4265-8DEC-A1CDB6675747}" name="crime" displayName="crime" ref="A1:D5" totalsRowShown="0" headerRowDxfId="67" headerRowBorderDxfId="66" tableBorderDxfId="65" totalsRowBorderDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EF810BE9-7C6F-4265-8DEC-A1CDB6675747}" name="crime" displayName="crime" ref="A1:D5" totalsRowShown="0" headerRowDxfId="71" headerRowBorderDxfId="70" tableBorderDxfId="69" totalsRowBorderDxfId="68">
   <autoFilter ref="A1:D5" xr:uid="{EF810BE9-7C6F-4265-8DEC-A1CDB6675747}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{907E3F67-1965-41D5-8DDD-707389C0597D}" name="Category" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{02A1EC8D-CE03-4112-AF55-3E5058D292AE}" name="Rate per 1,000" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{C292AD1E-37A6-4421-A549-FB7A56194F0B}" name="Cost per incident" dataDxfId="61"/>
-    <tableColumn id="4" xr3:uid="{7F206B66-30F3-4010-AC15-A9AFDE66E061}" name="Reduction rate" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{907E3F67-1965-41D5-8DDD-707389C0597D}" name="Category" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{02A1EC8D-CE03-4112-AF55-3E5058D292AE}" name="Rate per 1,000" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{C292AD1E-37A6-4421-A549-FB7A56194F0B}" name="Cost per incident" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{7F206B66-30F3-4010-AC15-A9AFDE66E061}" name="Reduction rate" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{55D7EC45-CE5C-44FC-B5E0-0BAFE887560C}" name="economic_coeff" displayName="economic_coeff" ref="A1:C8" totalsRowShown="0" headerRowDxfId="59" headerRowBorderDxfId="58" tableBorderDxfId="57" totalsRowBorderDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{55D7EC45-CE5C-44FC-B5E0-0BAFE887560C}" name="economic_coeff" displayName="economic_coeff" ref="A1:C8" totalsRowShown="0" headerRowDxfId="63" headerRowBorderDxfId="62" tableBorderDxfId="61" totalsRowBorderDxfId="60">
   <autoFilter ref="A1:C8" xr:uid="{55D7EC45-CE5C-44FC-B5E0-0BAFE887560C}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B3E4FC91-3B70-4B5F-BE4B-3D95311501D9}" name="Parameter" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{8E11059B-045B-4658-BEA4-ACFA568B296F}" name="Value" dataDxfId="54"/>
-    <tableColumn id="3" xr3:uid="{97CBA549-19DB-408B-AA6F-BDFA09076EB0}" name="Units" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{B3E4FC91-3B70-4B5F-BE4B-3D95311501D9}" name="Parameter" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{8E11059B-045B-4658-BEA4-ACFA568B296F}" name="Value" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{97CBA549-19DB-408B-AA6F-BDFA09076EB0}" name="Units" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7669,18 +7665,18 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="23">
-        <v>8.3333000000000001E-3</v>
+      <c r="B4" s="65">
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="C4" s="23">
-        <v>1.666666E-3</v>
+        <v>3.3E-3</v>
       </c>
       <c r="D4" s="23">
-        <v>3.3E-3</v>
+        <v>6.6E-3</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>70</v>

</xml_diff>